<commit_message>
Scope branch to Phase-1 showcase: drop legacy/pilot assets
Keep only the three-hop Phase-1 pipeline (CSV -> stage -> IL ->
consumption) plus shared framework internals. Remove Webster/Santander
and Bank1->MSS demo assets, pilot suites/contracts/fixtures, adapter
smoke scripts, and stale docs/images. Rewire defaults and CI to the
phase1 env/workbook pairs; load_phase2_hop gets a --hop shortcut.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/mapping/phase1_hop2_stage_to_il.xlsx
+++ b/data/mapping/phase1_hop2_stage_to_il.xlsx
@@ -1916,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1988,12 +1988,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dim_customer_address_migration</t>
+          <t>dim_customer_migration</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>dim_address_rows</t>
+          <t>dim_customer_by_type</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2002,10 +2002,14 @@
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>customer_type_cd</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dim_address_rows</t>
+          <t>dim_customer_by_type</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2017,12 +2021,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>dim_reference_migration</t>
+          <t>dim_customer_address_migration</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>dim_ref_rows</t>
+          <t>dim_address_rows</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2034,10 +2038,39 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
+          <t>dim_address_rows</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dim_reference_migration</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>dim_ref_rows</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>dim_ref_rows</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>